<commit_message>
DHT22 sensor interface included
</commit_message>
<xml_diff>
--- a/Documents/Safeflame_Product Backlog_Rithika.xlsx
+++ b/Documents/Safeflame_Product Backlog_Rithika.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\GitHub\SafeFlame\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FAD885F-9AD9-4090-B1EA-EED4400F5B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EC321C-32C0-42DF-B630-59816D6F37E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -923,7 +923,7 @@
         <v>3</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="29.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -974,7 +974,7 @@
         <v>3</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
New .c and .h file
LCD module was integrated to display weight and leak staus
</commit_message>
<xml_diff>
--- a/Documents/Safeflame_Product Backlog_Rithika.xlsx
+++ b/Documents/Safeflame_Product Backlog_Rithika.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\GitHub\SafeFlame\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C80C52-6C0A-45A1-90D2-24520DBB5491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B462E229-0C88-4E33-B710-B198AD103B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="80">
   <si>
     <t>Sprint</t>
   </si>
@@ -241,9 +241,6 @@
     <t>US21</t>
   </si>
   <si>
-    <t>US22</t>
-  </si>
-  <si>
     <t>Debug load cell code since load cell value is not printing every 1 second as per the delay added in the program.</t>
   </si>
   <si>
@@ -254,9 +251,6 @@
   </si>
   <si>
     <t>Interface LCD monitor using I2C for displaying output data</t>
-  </si>
-  <si>
-    <t>4-wire load cell need to be procured .Currently the 3 wire load cell is causing drift in reading without any weight.</t>
   </si>
   <si>
     <t>US24</t>
@@ -999,7 +993,7 @@
         <v>3</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="L13" s="2"/>
     </row>
@@ -1132,7 +1126,7 @@
         <v>3</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -1146,7 +1140,7 @@
         <v>66</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="3" t="s">
@@ -1173,7 +1167,7 @@
         <v>69</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="3" t="s">
@@ -1213,7 +1207,7 @@
         <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -1227,7 +1221,7 @@
         <v>72</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="3" t="s">
@@ -1248,13 +1242,13 @@
         <v>53</v>
       </c>
       <c r="B23" s="3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="3" t="s">
@@ -1264,10 +1258,10 @@
         <v>5</v>
       </c>
       <c r="H23" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -1275,23 +1269,23 @@
         <v>53</v>
       </c>
       <c r="B24" s="3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G24" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H24" s="3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>15</v>
@@ -1302,54 +1296,30 @@
         <v>53</v>
       </c>
       <c r="B25" s="3">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G25" s="3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H25" s="3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="22.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" s="3">
-        <v>25</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="3">
-        <v>3</v>
-      </c>
-      <c r="H26" s="3">
-        <v>3</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="A26" s="2"/>
       <c r="J26" s="3"/>
     </row>
     <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2634,13 +2604,13 @@
     <mergeCell ref="B54:C54"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F42:F44 F2:F40" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F42:F44 F2:F25 F27:F40" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$L$3:$L$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I42:I50 I2:I40" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I42:I50 I2:I25 I27:I40" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>$N$3:$N$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E42:E50 E17:E40 E13 E2:E11" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E42:E50 E13 E2:E11 E17:E25 E27:E40" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>$L$10:$L$14</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
GSM source code updated
rx buffer size was updated
</commit_message>
<xml_diff>
--- a/Documents/Safeflame_Product Backlog_Rithika.xlsx
+++ b/Documents/Safeflame_Product Backlog_Rithika.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\GitHub\SafeFlame\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6185EBF-DC59-4D8D-A318-F6FACBAD5728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3535764F-F98C-4906-85FF-FBF593AFA58C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1243,7 +1243,7 @@
         <v>4</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -1270,7 +1270,7 @@
         <v>7</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -1324,7 +1324,7 @@
         <v>2</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J25" s="3"/>
     </row>
@@ -1352,7 +1352,7 @@
         <v>4</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>